<commit_message>
importation arab fixed need testing
</commit_message>
<xml_diff>
--- a/importationFileUpload/Template-hhhhhhhhhhhhhh-Ar.xlsx
+++ b/importationFileUpload/Template-hhhhhhhhhhhhhh-Ar.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27531"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Houda\Documents\SDL3\sourceEnq\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\develepement\SDL3\importationFileUpload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07CB4846-E6FA-4ACE-B957-233B0599E5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Arabe" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Arabe!$A$1:$AC$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Arabe!$A$1:$AE$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>العدد</t>
   </si>
@@ -91,22 +90,6 @@
   </si>
   <si>
     <t>لقـــب أم الــزوج(ة)</t>
-  </si>
-  <si>
-    <t>مستوى
-المداخيل</t>
-  </si>
-  <si>
-    <t>ظروف
-السكن</t>
-  </si>
-  <si>
-    <t>الحالة
-العائلية</t>
-  </si>
-  <si>
-    <t>أقدمية
-طلب السكن</t>
   </si>
   <si>
     <t>المجموع</t>
@@ -216,13 +199,28 @@
       <t>)</t>
     </r>
   </si>
+  <si>
+    <t>عدد الزوجات</t>
+  </si>
+  <si>
+    <t>ترتيب الزوجة</t>
+  </si>
+  <si>
+    <t>مستوى المداخيل</t>
+  </si>
+  <si>
+    <t>ظروف السكن</t>
+  </si>
+  <si>
+    <t>أقدمية طلب السكن</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -422,7 +420,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyFont="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyFont="0">
       <alignment horizontal="center"/>
@@ -464,18 +462,18 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="12">
-    <cellStyle name="Currency" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="Currency 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Currency" xfId="5"/>
+    <cellStyle name="Currency 2" xfId="9"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 2 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Normal 2 4" xfId="10" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Style 1" xfId="2" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Style 2" xfId="8" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Style 2 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="Style 6" xfId="4" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Normal 2" xfId="6"/>
+    <cellStyle name="Normal 2 2" xfId="7"/>
+    <cellStyle name="Normal 2 3" xfId="1"/>
+    <cellStyle name="Normal 2 4" xfId="10"/>
+    <cellStyle name="Normal 3" xfId="3"/>
+    <cellStyle name="Style 1" xfId="2"/>
+    <cellStyle name="Style 2" xfId="8"/>
+    <cellStyle name="Style 2 2" xfId="11"/>
+    <cellStyle name="Style 6" xfId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -752,43 +750,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:AC15"/>
+  <dimension ref="A1:AE15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="51.85546875" customWidth="1"/>
-    <col min="15" max="15" width="24.85546875" customWidth="1"/>
-    <col min="16" max="16" width="22.28515625" customWidth="1"/>
-    <col min="17" max="17" width="26" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="34.85546875" customWidth="1"/>
-    <col min="20" max="20" width="34.7109375" customWidth="1"/>
-    <col min="21" max="21" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="31.42578125" customWidth="1"/>
-    <col min="24" max="24" width="17" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="22.42578125" customWidth="1"/>
-    <col min="27" max="27" width="34.7109375" customWidth="1"/>
-    <col min="28" max="28" width="23.140625" customWidth="1"/>
-    <col min="29" max="29" width="47.5703125" customWidth="1"/>
+    <col min="3" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="51.85546875" customWidth="1"/>
+    <col min="17" max="17" width="24.85546875" customWidth="1"/>
+    <col min="18" max="18" width="22.28515625" customWidth="1"/>
+    <col min="19" max="19" width="26" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="34.85546875" customWidth="1"/>
+    <col min="22" max="22" width="34.7109375" customWidth="1"/>
+    <col min="23" max="23" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.42578125" customWidth="1"/>
+    <col min="26" max="26" width="18.28515625" customWidth="1"/>
+    <col min="27" max="27" width="16" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="22.42578125" customWidth="1"/>
+    <col min="29" max="29" width="34.7109375" customWidth="1"/>
+    <col min="30" max="30" width="23.140625" customWidth="1"/>
+    <col min="31" max="31" width="47.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="1" customFormat="1" ht="54" thickTop="1" thickBot="1">
+    <row r="1" spans="1:31" s="1" customFormat="1" ht="54" thickTop="1" thickBot="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -798,86 +796,92 @@
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="U1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="V1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="Y1" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="U1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="W1" s="10" t="s">
+      <c r="AA1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="AB1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="AE1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="Z1" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="AB1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="AC1" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" s="12" customFormat="1" ht="27.75" thickTop="1" thickBot="1">
+    </row>
+    <row r="2" spans="1:31" s="12" customFormat="1" ht="27.75" thickTop="1" thickBot="1">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -907,8 +911,10 @@
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AC2" s="3"/>
-    </row>
-    <row r="3" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="3"/>
+    </row>
+    <row r="3" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -938,8 +944,10 @@
       <c r="AA3" s="3"/>
       <c r="AB3" s="3"/>
       <c r="AC3" s="3"/>
-    </row>
-    <row r="4" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+    </row>
+    <row r="4" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -969,8 +977,10 @@
       <c r="AA4" s="3"/>
       <c r="AB4" s="3"/>
       <c r="AC4" s="3"/>
-    </row>
-    <row r="5" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+    </row>
+    <row r="5" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1000,8 +1010,10 @@
       <c r="AA5" s="3"/>
       <c r="AB5" s="3"/>
       <c r="AC5" s="3"/>
-    </row>
-    <row r="6" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD5" s="3"/>
+      <c r="AE5" s="3"/>
+    </row>
+    <row r="6" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1031,8 +1043,10 @@
       <c r="AA6" s="3"/>
       <c r="AB6" s="3"/>
       <c r="AC6" s="3"/>
-    </row>
-    <row r="7" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD6" s="3"/>
+      <c r="AE6" s="3"/>
+    </row>
+    <row r="7" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -1062,8 +1076,10 @@
       <c r="AA7" s="3"/>
       <c r="AB7" s="3"/>
       <c r="AC7" s="3"/>
-    </row>
-    <row r="8" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD7" s="3"/>
+      <c r="AE7" s="3"/>
+    </row>
+    <row r="8" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -1093,8 +1109,10 @@
       <c r="AA8" s="3"/>
       <c r="AB8" s="3"/>
       <c r="AC8" s="3"/>
-    </row>
-    <row r="9" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+    </row>
+    <row r="9" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -1124,8 +1142,10 @@
       <c r="AA9" s="3"/>
       <c r="AB9" s="3"/>
       <c r="AC9" s="3"/>
-    </row>
-    <row r="10" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD9" s="3"/>
+      <c r="AE9" s="3"/>
+    </row>
+    <row r="10" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -1155,8 +1175,10 @@
       <c r="AA10" s="3"/>
       <c r="AB10" s="3"/>
       <c r="AC10" s="3"/>
-    </row>
-    <row r="11" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD10" s="3"/>
+      <c r="AE10" s="3"/>
+    </row>
+    <row r="11" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -1186,8 +1208,10 @@
       <c r="AA11" s="3"/>
       <c r="AB11" s="3"/>
       <c r="AC11" s="3"/>
-    </row>
-    <row r="12" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD11" s="3"/>
+      <c r="AE11" s="3"/>
+    </row>
+    <row r="12" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -1217,8 +1241,10 @@
       <c r="AA12" s="3"/>
       <c r="AB12" s="3"/>
       <c r="AC12" s="3"/>
-    </row>
-    <row r="13" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD12" s="3"/>
+      <c r="AE12" s="3"/>
+    </row>
+    <row r="13" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1248,8 +1274,10 @@
       <c r="AA13" s="3"/>
       <c r="AB13" s="3"/>
       <c r="AC13" s="3"/>
-    </row>
-    <row r="14" spans="1:29" ht="27.75" thickTop="1" thickBot="1">
+      <c r="AD13" s="3"/>
+      <c r="AE13" s="3"/>
+    </row>
+    <row r="14" spans="1:31" ht="27.75" thickTop="1" thickBot="1">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1279,8 +1307,10 @@
       <c r="AA14" s="3"/>
       <c r="AB14" s="3"/>
       <c r="AC14" s="3"/>
-    </row>
-    <row r="15" spans="1:29" ht="27" thickTop="1">
+      <c r="AD14" s="3"/>
+      <c r="AE14" s="3"/>
+    </row>
+    <row r="15" spans="1:31" ht="27" thickTop="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -1310,10 +1340,12 @@
       <c r="AA15" s="3"/>
       <c r="AB15" s="3"/>
       <c r="AC15" s="3"/>
+      <c r="AD15" s="3"/>
+      <c r="AE15" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC1" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC86">
+  <autoFilter ref="A1:AE1">
+    <sortState ref="A2:AC86">
       <sortCondition ref="C1"/>
     </sortState>
   </autoFilter>

</xml_diff>